<commit_message>
Update intent test case spreadsheets
Updates to main and Jack's intent test case workbooks.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Cidy_Intent_Test_Cases_90.xlsx
+++ b/documentation/Cidy_Intent_Test_Cases_90.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RRAPOPOR\Documents\Cidy testing\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{037A6EC7-7F7D-4DD3-9197-E75306B8ED71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B321AE45-2C33-49A0-828E-D8E5D31AD937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="303">
   <si>
     <t>Scenario</t>
   </si>
@@ -152,28 +152,7 @@
     <t>Routes directly to Programme Development with topic_area=projects_evaluations. This is actual evaluation evidence, not evaluation design guidance.</t>
   </si>
   <si>
-    <t>Happy path - evaluation recommendations</t>
-  </si>
-  <si>
-    <t>Summarize recommendations from project evaluations related to stakeholder engagement.</t>
-  </si>
-  <si>
     <t>Routes to Programme Development with topic_area=projects_evaluations.</t>
-  </si>
-  <si>
-    <t>Happy path - lessons learned</t>
-  </si>
-  <si>
-    <t>What lessons learned are available from past capacity development projects?</t>
-  </si>
-  <si>
-    <t>Happy path - DA evaluation evidence distinction</t>
-  </si>
-  <si>
-    <t>What have evaluations said about DA projects?</t>
-  </si>
-  <si>
-    <t>Routes to Programme Development with topic_area=projects_evaluations, using DA as context if available. It should not route to DA evaluation design guidance.</t>
   </si>
   <si>
     <t>Happy path - recurring evaluation findings</t>
@@ -1127,14 +1106,49 @@
     <t>CorrectSources</t>
   </si>
   <si>
-    <t xml:space="preserve">Answer: I was not able to find information in my knowledge sources that could answer this question.
+    <t>Cidy is designed to support DESA capacity-development knowledge, including DA, RPTC, UNPDF/PDF, Programme Development, Project Evaluation evidence, and Cidy-related guidance. This question appears outside that scope.</t>
+  </si>
+  <si>
+    <t>Answer: Yes, several recurring findings and common themes have been identified in past project evaluations within DESA capacity development projects:
+Importance of Policy Engagement and Stakeholder Involvement
+Prioritising policy engagement is often highlighted as a primary pathway to scale project impact.
+Continued engagement with policymakers and entrepreneurs is essential for the uptake and sustainability of project outcomes.
+Involving political decision-makers from the beginning and maintaining permanent policy dialogue is recommended.
+Adaptive and Outcome-Focused Project Design
+Projects benefit from adaptive, demand-driven capacity building and outcome-focused, indicator-based monitoring and follow-up systems.
+Overambitious project designs can limit delivery under constrained resources, and missed monitoring opportunities can limit evidence of results.
+Capacity Building and Methodological Transfer
+Joint and integrated modelling and training work contribute to effective methodological transfer.
+Achieving integrated assessment of development dimensions requires addressing technical, political-strategic, and organizational challenges simultaneously.
+Sustainability and Collaboration
+Sustainability is enhanced by involving influential community members and building capacity.
+Permanent collaboration mechanisms with public institutions and national universities are important for long-term impact.
+Lessons Learned
+Drafting policies alone is not sufficient; continued engagement and operationalisation of policy products are necessary.
+Convening policymakers and entrepreneurs, as well as adaptive project management, are effective strategies.
+Different strategies exist to leave capacities installed in beneficiary countries, each with its own pros and cons.
+These themes are consistently reflected in evaluation reports and lessons learned sections across multiple projects and years, including those focused on MSME resilience, integrated modelling tools, and sustainable development policy support.
 Sources:
-No sources found.
-Confidence: Low
- </t>
-  </si>
-  <si>
-    <t>Cidy is designed to support DESA capacity-development knowledge, including DA, RPTC, UNPDF/PDF, Programme Development, Project Evaluation evidence, and Cidy-related guidance. This question appears outside that scope.</t>
+Evaluations Log Static File.xlsx
+Confidence: Very High</t>
+  </si>
+  <si>
+    <t>Required Fix</t>
+  </si>
+  <si>
+    <t>Answer: Evaluation reports and final report templates for UN Development Account projects recommend that weaknesses in project design should be explicitly addressed in the section on challenges or problems encountered. Project managers are asked to elaborate on issues related to the project’s design, such as the type of outputs, outcomes, objectives, and any significant variations from the original project plan. These weaknesses may include:
+Inadequate or unclear objectives and outcomes.
+Outputs that do not sufficiently contribute to the intended outcomes.
+Faulty assumptions in the theory of change or logical framework.
+Insufficient integration of gender, human rights, or the principle of “leaving no one behind.”
+Gaps in stakeholder engagement or capacity assessment.
+Lack of alignment with national or regional frameworks.
+Poorly defined indicators or means of verification.
+Evaluation reports also encourage documenting actions taken to address these weaknesses and highlight lessons learned for future programming. Good practices and innovative approaches that successfully addressed design weaknesses should be shared, and the sustainability of project achievements should be considered in the design phase to avoid weaknesses that could undermine long-term impact. These insights are typically captured in dedicated tables or narrative sections within the final report template, ensuring systematic institutional learning and accountability for project design quality.
+Sources:
+generic_project_document_guidelines_final.docx
+project_final_report_0.docx
+Confidence: High</t>
   </si>
 </sst>
 </file>
@@ -1195,20 +1209,25 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="17">
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -1299,13 +1318,6 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1469,20 +1481,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TestCases" displayName="TestCases" ref="A1:K101" headerRowDxfId="18" dataDxfId="12" totalsRowDxfId="17">
-  <autoFilter ref="A1:K101" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Scenario" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Test Question" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{68F948D1-0E8A-4480-8723-80EC07BAA04C}" name="Prod Answer" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{FC7C6CC2-66C4-4B78-8F9E-DC4824CA4968}" name="FoundAnswer" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{551CDDA9-7BAE-4AE5-8237-BD7504F9E735}" name="AnswerQuality" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{EC4A9B6F-8976-43CC-A78B-D4C6C117B8BA}" name="CorrectSources" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{30840C4C-93AB-4657-A3EE-B277ADF5F742}" name="Test Date" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{DB32ACFF-3AD3-4851-952B-2F2090D84F8D}" name="Perfomance" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Clarification" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Expected Behavior" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Date Created" dataDxfId="13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TestCases" displayName="TestCases" ref="A1:L98" headerRowDxfId="16" dataDxfId="10" totalsRowDxfId="15">
+  <autoFilter ref="A1:L98" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Scenario" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Test Question" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{68F948D1-0E8A-4480-8723-80EC07BAA04C}" name="Prod Answer" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{FC7C6CC2-66C4-4B78-8F9E-DC4824CA4968}" name="FoundAnswer" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{551CDDA9-7BAE-4AE5-8237-BD7504F9E735}" name="AnswerQuality" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{EC4A9B6F-8976-43CC-A78B-D4C6C117B8BA}" name="CorrectSources" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{8AF5338E-8524-4734-9FCB-D3197EB1FB54}" name="Required Fix" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{30840C4C-93AB-4657-A3EE-B277ADF5F742}" name="Test Date" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{DB32ACFF-3AD3-4851-952B-2F2090D84F8D}" name="Perfomance" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Clarification" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Expected Behavior" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Date Created" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1806,21 +1819,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.453125" style="4" customWidth="1"/>
     <col min="2" max="2" width="32.26953125" style="4" customWidth="1"/>
     <col min="3" max="3" width="32.26953125" style="5" customWidth="1"/>
-    <col min="4" max="6" width="12.90625" style="4" customWidth="1"/>
-    <col min="7" max="8" width="9.7265625" style="4" customWidth="1"/>
-    <col min="9" max="9" width="17.81640625" style="3" customWidth="1"/>
-    <col min="10" max="10" width="286" style="3" customWidth="1"/>
-    <col min="11" max="11" width="15.453125" style="3" customWidth="1"/>
-    <col min="12" max="16384" width="8.7265625" style="3"/>
+    <col min="4" max="7" width="12.90625" style="4" customWidth="1"/>
+    <col min="8" max="9" width="9.7265625" style="4" customWidth="1"/>
+    <col min="10" max="10" width="17.81640625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="286" style="3" customWidth="1"/>
+    <col min="12" max="12" width="15.453125" style="3" customWidth="1"/>
+    <col min="13" max="16384" width="8.7265625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1828,34 +1841,37 @@
         <v>1</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
@@ -1863,29 +1879,29 @@
         <v>6</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="H2" s="7">
+        <v>46184</v>
+      </c>
+      <c r="I2" s="7" t="s">
         <v>290</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>293</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="G2" s="7">
-        <v>46184</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>297</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>7</v>
-      </c>
       <c r="J2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="5"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L2" s="5"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>9</v>
       </c>
@@ -1893,29 +1909,29 @@
         <v>10</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="G3" s="7">
+        <v>286</v>
+      </c>
+      <c r="H3" s="7">
         <v>46184</v>
       </c>
-      <c r="H3" s="7" t="s">
-        <v>297</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>7</v>
+      <c r="I3" s="7" t="s">
+        <v>290</v>
       </c>
       <c r="J3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="5"/>
-    </row>
-    <row r="4" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L3" s="5"/>
+    </row>
+    <row r="4" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>12</v>
       </c>
@@ -1923,26 +1939,26 @@
         <v>13</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="G4" s="7">
+        <v>292</v>
+      </c>
+      <c r="H4" s="7">
         <v>46184</v>
       </c>
-      <c r="H4" s="7" t="s">
-        <v>297</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>7</v>
+      <c r="I4" s="7" t="s">
+        <v>290</v>
       </c>
       <c r="J4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="5"/>
-    </row>
-    <row r="5" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L4" s="5"/>
+    </row>
+    <row r="5" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>15</v>
       </c>
@@ -1950,27 +1966,27 @@
         <v>16</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="G5" s="7">
+        <v>286</v>
+      </c>
+      <c r="H5" s="7">
         <v>46184</v>
       </c>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I5" s="5"/>
       <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="5"/>
-    </row>
-    <row r="6" spans="1:11" ht="60" x14ac:dyDescent="0.3">
+      <c r="L5" s="5"/>
+    </row>
+    <row r="6" spans="1:12" ht="60" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>18</v>
       </c>
@@ -1978,24 +1994,24 @@
         <v>19</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="G6" s="7">
+        <v>292</v>
+      </c>
+      <c r="H6" s="7">
         <v>46184</v>
       </c>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I6" s="5"/>
       <c r="J6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="K6" s="5"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L6" s="5"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>21</v>
       </c>
@@ -2003,27 +2019,27 @@
         <v>22</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="G7" s="7">
+        <v>286</v>
+      </c>
+      <c r="H7" s="7">
         <v>46184</v>
       </c>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I7" s="5"/>
       <c r="J7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K7" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="K7" s="5"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L7" s="5"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>24</v>
       </c>
@@ -2031,27 +2047,27 @@
         <v>25</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="G8" s="7">
+        <v>286</v>
+      </c>
+      <c r="H8" s="7">
         <v>46184</v>
       </c>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I8" s="5"/>
       <c r="J8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K8" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="K8" s="5"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L8" s="5"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>27</v>
       </c>
@@ -2059,27 +2075,27 @@
         <v>28</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="G9" s="7">
+        <v>286</v>
+      </c>
+      <c r="H9" s="7">
         <v>46184</v>
       </c>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I9" s="5"/>
       <c r="J9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K9" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="K9" s="5"/>
-    </row>
-    <row r="10" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L9" s="5"/>
+    </row>
+    <row r="10" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>30</v>
       </c>
@@ -2087,27 +2103,27 @@
         <v>31</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>299</v>
-      </c>
-      <c r="G10" s="7">
+        <v>292</v>
+      </c>
+      <c r="H10" s="7">
         <v>46184</v>
       </c>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I10" s="5"/>
       <c r="J10" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K10" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="K10" s="5"/>
-    </row>
-    <row r="11" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L10" s="5"/>
+    </row>
+    <row r="11" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>33</v>
       </c>
@@ -2115,25 +2131,25 @@
         <v>34</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="G11" s="5"/>
+        <v>286</v>
+      </c>
       <c r="H11" s="5"/>
-      <c r="I11" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I11" s="5"/>
       <c r="J11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K11" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="K11" s="5"/>
-    </row>
-    <row r="12" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L11" s="5"/>
+    </row>
+    <row r="12" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>36</v>
       </c>
@@ -2141,40 +2157,48 @@
         <v>37</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="G12" s="5"/>
+        <v>292</v>
+      </c>
       <c r="H12" s="5"/>
-      <c r="I12" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I12" s="5"/>
       <c r="J12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K12" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="K12" s="5"/>
-    </row>
-    <row r="13" spans="1:11" ht="36" x14ac:dyDescent="0.3">
+      <c r="L12" s="5"/>
+    </row>
+    <row r="13" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K13" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J13" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="K13" s="5"/>
-    </row>
-    <row r="14" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L13" s="5"/>
+    </row>
+    <row r="14" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>42</v>
       </c>
@@ -2182,22 +2206,20 @@
         <v>43</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>306</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="G14" s="5"/>
+        <v>302</v>
+      </c>
+      <c r="D14" s="5"/>
       <c r="H14" s="5"/>
-      <c r="I14" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I14" s="5"/>
       <c r="J14" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="K14" s="5"/>
-    </row>
-    <row r="15" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L14" s="5"/>
+    </row>
+    <row r="15" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>44</v>
       </c>
@@ -2205,53 +2227,53 @@
         <v>45</v>
       </c>
       <c r="D15" s="5"/>
-      <c r="G15" s="5"/>
       <c r="H15" s="5"/>
-      <c r="I15" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I15" s="5"/>
       <c r="J15" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L15" s="5"/>
+    </row>
+    <row r="16" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="K15" s="5"/>
-    </row>
-    <row r="16" spans="1:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="D16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L16" s="5"/>
+    </row>
+    <row r="17" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="K16" s="5"/>
-    </row>
-    <row r="17" spans="1:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="D17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K17" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J17" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="K17" s="5"/>
-    </row>
-    <row r="18" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L17" s="5"/>
+    </row>
+    <row r="18" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>51</v>
       </c>
@@ -2259,107 +2281,107 @@
         <v>52</v>
       </c>
       <c r="D18" s="5"/>
-      <c r="G18" s="5"/>
       <c r="H18" s="5"/>
-      <c r="I18" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I18" s="5"/>
       <c r="J18" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="K18" s="5"/>
-    </row>
-    <row r="19" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="L18" s="5"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D19" s="5"/>
-      <c r="G19" s="5"/>
       <c r="H19" s="5"/>
-      <c r="I19" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I19" s="5"/>
       <c r="J19" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="K19" s="5"/>
-    </row>
-    <row r="20" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="L19" s="5"/>
+    </row>
+    <row r="20" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D20" s="5"/>
-      <c r="G20" s="5"/>
       <c r="H20" s="5"/>
-      <c r="I20" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I20" s="5"/>
       <c r="J20" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="K20" s="5"/>
-    </row>
-    <row r="21" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K20" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="L20" s="5"/>
+    </row>
+    <row r="21" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D21" s="5"/>
-      <c r="G21" s="5"/>
       <c r="H21" s="5"/>
-      <c r="I21" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I21" s="5"/>
       <c r="J21" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="K21" s="5"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K21" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="L21" s="5"/>
+    </row>
+    <row r="22" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B22" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K22" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J22" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="K22" s="5"/>
-    </row>
-    <row r="23" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L22" s="5"/>
+    </row>
+    <row r="23" spans="1:12" ht="36" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D23" s="5"/>
-      <c r="G23" s="5"/>
       <c r="H23" s="5"/>
-      <c r="I23" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I23" s="5"/>
       <c r="J23" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="K23" s="5"/>
-    </row>
-    <row r="24" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="L23" s="5"/>
+    </row>
+    <row r="24" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>67</v>
       </c>
@@ -2367,17 +2389,17 @@
         <v>68</v>
       </c>
       <c r="D24" s="5"/>
-      <c r="G24" s="5"/>
       <c r="H24" s="5"/>
-      <c r="I24" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I24" s="5"/>
       <c r="J24" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K24" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="K24" s="5"/>
-    </row>
-    <row r="25" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L24" s="5"/>
+    </row>
+    <row r="25" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>70</v>
       </c>
@@ -2385,17 +2407,17 @@
         <v>71</v>
       </c>
       <c r="D25" s="5"/>
-      <c r="G25" s="5"/>
       <c r="H25" s="5"/>
-      <c r="I25" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I25" s="5"/>
       <c r="J25" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K25" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="K25" s="5"/>
-    </row>
-    <row r="26" spans="1:11" ht="36" x14ac:dyDescent="0.3">
+      <c r="L25" s="5"/>
+    </row>
+    <row r="26" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>72</v>
       </c>
@@ -2403,17 +2425,17 @@
         <v>73</v>
       </c>
       <c r="D26" s="5"/>
-      <c r="G26" s="5"/>
       <c r="H26" s="5"/>
-      <c r="I26" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I26" s="5"/>
       <c r="J26" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K26" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="K26" s="5"/>
-    </row>
-    <row r="27" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L26" s="5"/>
+    </row>
+    <row r="27" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>74</v>
       </c>
@@ -2421,17 +2443,17 @@
         <v>75</v>
       </c>
       <c r="D27" s="5"/>
-      <c r="G27" s="5"/>
       <c r="H27" s="5"/>
-      <c r="I27" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I27" s="5"/>
       <c r="J27" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K27" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="K27" s="5"/>
-    </row>
-    <row r="28" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L27" s="5"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>77</v>
       </c>
@@ -2439,17 +2461,17 @@
         <v>78</v>
       </c>
       <c r="D28" s="5"/>
-      <c r="G28" s="5"/>
       <c r="H28" s="5"/>
-      <c r="I28" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I28" s="5"/>
       <c r="J28" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K28" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="K28" s="5"/>
-    </row>
-    <row r="29" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L28" s="5"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>79</v>
       </c>
@@ -2457,17 +2479,17 @@
         <v>80</v>
       </c>
       <c r="D29" s="5"/>
-      <c r="G29" s="5"/>
       <c r="H29" s="5"/>
-      <c r="I29" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I29" s="5"/>
       <c r="J29" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K29" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="K29" s="5"/>
-    </row>
-    <row r="30" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L29" s="5"/>
+    </row>
+    <row r="30" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>81</v>
       </c>
@@ -2475,71 +2497,71 @@
         <v>82</v>
       </c>
       <c r="D30" s="5"/>
-      <c r="G30" s="5"/>
       <c r="H30" s="5"/>
-      <c r="I30" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I30" s="5"/>
       <c r="J30" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K30" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L30" s="5"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A31" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="K30" s="5"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
+      <c r="B31" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="D31" s="5"/>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5"/>
+      <c r="J31" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K31" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L31" s="5"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A32" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D31" s="5"/>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J31" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="K31" s="5"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A32" s="5" t="s">
+      <c r="B32" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="D32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L32" s="5"/>
+    </row>
+    <row r="33" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D32" s="5"/>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J32" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="K32" s="5"/>
-    </row>
-    <row r="33" spans="1:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="A33" s="5" t="s">
+      <c r="B33" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="D33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K33" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="D33" s="5"/>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J33" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="K33" s="5"/>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L33" s="5"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>90</v>
       </c>
@@ -2547,601 +2569,605 @@
         <v>91</v>
       </c>
       <c r="D34" s="5"/>
-      <c r="G34" s="5"/>
       <c r="H34" s="5"/>
-      <c r="I34" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I34" s="5"/>
       <c r="J34" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="K34" s="5"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K34" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="L34" s="5"/>
+    </row>
+    <row r="35" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D35" s="5"/>
-      <c r="G35" s="5"/>
       <c r="H35" s="5"/>
-      <c r="I35" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I35" s="5"/>
       <c r="J35" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="K35" s="5"/>
-    </row>
-    <row r="36" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="L35" s="5"/>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B36" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D36" s="5"/>
+      <c r="H36" s="5"/>
+      <c r="I36" s="5"/>
+      <c r="J36" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K36" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="D36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J36" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="K36" s="5"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L36" s="5"/>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D37" s="5"/>
-      <c r="G37" s="5"/>
       <c r="H37" s="5"/>
-      <c r="I37" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I37" s="5"/>
       <c r="J37" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="K37" s="5"/>
-    </row>
-    <row r="38" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+      <c r="K37" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="L37" s="5"/>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D38" s="5"/>
+      <c r="H38" s="5"/>
+      <c r="I38" s="5"/>
+      <c r="J38" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="K38" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="L38" s="5"/>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A39" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D39" s="5"/>
+      <c r="H39" s="5"/>
+      <c r="I39" s="5"/>
+      <c r="J39" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="K39" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="L39" s="5"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A40" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D40" s="5"/>
+      <c r="H40" s="5"/>
+      <c r="I40" s="5"/>
+      <c r="J40" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="K40" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="L40" s="5"/>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A41" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D41" s="5"/>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="B38" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D38" s="5"/>
-      <c r="G38" s="5"/>
-      <c r="H38" s="5"/>
-      <c r="I38" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J38" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="K38" s="5"/>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A39" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="B39" s="4" t="s">
+      <c r="K41" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="L41" s="5"/>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A42" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D42" s="5"/>
+      <c r="H42" s="5"/>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="K42" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="L42" s="5"/>
+    </row>
+    <row r="43" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A43" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D43" s="5"/>
+      <c r="H43" s="5"/>
+      <c r="I43" s="5"/>
+      <c r="J43" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="K43" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="L43" s="5"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D44" s="5"/>
+      <c r="H44" s="5"/>
+      <c r="I44" s="5"/>
+      <c r="J44" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="K44" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="L44" s="5"/>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A45" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D45" s="5"/>
+      <c r="H45" s="5"/>
+      <c r="I45" s="5"/>
+      <c r="J45" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D39" s="5"/>
-      <c r="G39" s="5"/>
-      <c r="H39" s="5"/>
-      <c r="I39" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J39" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="K39" s="5"/>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="D40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-      <c r="I40" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="J40" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="K40" s="5"/>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A41" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="D41" s="5"/>
-      <c r="G41" s="5"/>
-      <c r="H41" s="5"/>
-      <c r="I41" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="J41" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="K41" s="5"/>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A42" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="D42" s="5"/>
-      <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
-      <c r="I42" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="J42" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="K42" s="5"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A43" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="D43" s="5"/>
-      <c r="G43" s="5"/>
-      <c r="H43" s="5"/>
-      <c r="I43" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="J43" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="K43" s="5"/>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A44" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="D44" s="5"/>
-      <c r="G44" s="5"/>
-      <c r="H44" s="5"/>
-      <c r="I44" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="J44" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="K44" s="5"/>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A45" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="D45" s="5"/>
-      <c r="G45" s="5"/>
-      <c r="H45" s="5"/>
-      <c r="I45" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="J45" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="K45" s="5"/>
-    </row>
-    <row r="46" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="K45" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="L45" s="5"/>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D46" s="5"/>
-      <c r="G46" s="5"/>
       <c r="H46" s="5"/>
-      <c r="I46" s="5" t="s">
-        <v>129</v>
-      </c>
+      <c r="I46" s="5"/>
       <c r="J46" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="K46" s="5"/>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+        <v>133</v>
+      </c>
+      <c r="K46" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="L46" s="5"/>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>132</v>
       </c>
       <c r="D47" s="5"/>
-      <c r="G47" s="5"/>
       <c r="H47" s="5"/>
-      <c r="I47" s="5" t="s">
-        <v>133</v>
-      </c>
+      <c r="I47" s="5"/>
       <c r="J47" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="K47" s="5"/>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+      <c r="K47" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="L47" s="5"/>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D48" s="5"/>
-      <c r="G48" s="5"/>
       <c r="H48" s="5"/>
-      <c r="I48" s="5" t="s">
-        <v>111</v>
-      </c>
+      <c r="I48" s="5"/>
       <c r="J48" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="K48" s="5"/>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+      <c r="K48" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="L48" s="5"/>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D49" s="5"/>
-      <c r="G49" s="5"/>
       <c r="H49" s="5"/>
-      <c r="I49" s="5" t="s">
-        <v>140</v>
-      </c>
+      <c r="I49" s="5"/>
       <c r="J49" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="K49" s="5"/>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+      <c r="K49" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="L49" s="5"/>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="D50" s="5"/>
-      <c r="G50" s="5"/>
       <c r="H50" s="5"/>
-      <c r="I50" s="5" t="s">
-        <v>143</v>
-      </c>
+      <c r="I50" s="5"/>
       <c r="J50" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="K50" s="5"/>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+        <v>148</v>
+      </c>
+      <c r="K50" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="L50" s="5"/>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D51" s="5"/>
-      <c r="G51" s="5"/>
       <c r="H51" s="5"/>
-      <c r="I51" s="5" t="s">
-        <v>147</v>
-      </c>
+      <c r="I51" s="5"/>
       <c r="J51" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="K51" s="5"/>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+        <v>152</v>
+      </c>
+      <c r="K51" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="L51" s="5"/>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="D52" s="5"/>
-      <c r="G52" s="5"/>
       <c r="H52" s="5"/>
-      <c r="I52" s="5" t="s">
+      <c r="I52" s="5"/>
+      <c r="J52" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="K52" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="L52" s="5"/>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A53" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="D53" s="5"/>
+      <c r="H53" s="5"/>
+      <c r="I53" s="5"/>
+      <c r="J53" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="K53" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="L53" s="5"/>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A54" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="D54" s="5"/>
+      <c r="H54" s="5"/>
+      <c r="I54" s="5"/>
+      <c r="J54" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="K54" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="L54" s="5"/>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A55" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D55" s="5"/>
+      <c r="H55" s="5"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K55" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="L55" s="5"/>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A56" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="D56" s="5"/>
+      <c r="H56" s="5"/>
+      <c r="I56" s="5"/>
+      <c r="J56" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K56" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="L56" s="5"/>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A57" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="B57" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="J52" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="K52" s="5"/>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A53" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="D53" s="5"/>
-      <c r="G53" s="5"/>
-      <c r="H53" s="5"/>
-      <c r="I53" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="J53" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="K53" s="5"/>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A54" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="D54" s="5"/>
-      <c r="G54" s="5"/>
-      <c r="H54" s="5"/>
-      <c r="I54" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="J54" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="K54" s="5"/>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A55" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="D55" s="5"/>
-      <c r="G55" s="5"/>
-      <c r="H55" s="5"/>
-      <c r="I55" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="J55" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="K55" s="5"/>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A56" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="D56" s="5"/>
-      <c r="G56" s="5"/>
-      <c r="H56" s="5"/>
-      <c r="I56" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="J56" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="K56" s="5"/>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A57" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>166</v>
-      </c>
       <c r="D57" s="5"/>
-      <c r="G57" s="5"/>
       <c r="H57" s="5"/>
-      <c r="I57" s="5" t="s">
-        <v>170</v>
-      </c>
+      <c r="I57" s="5"/>
       <c r="J57" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="K57" s="5"/>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K57" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="L57" s="5"/>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D58" s="5"/>
-      <c r="G58" s="5"/>
       <c r="H58" s="5"/>
-      <c r="I58" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I58" s="5"/>
       <c r="J58" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="K58" s="5"/>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K58" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="L58" s="5"/>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D59" s="5"/>
-      <c r="G59" s="5"/>
       <c r="H59" s="5"/>
-      <c r="I59" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I59" s="5"/>
       <c r="J59" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="K59" s="5"/>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K59" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="L59" s="5"/>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="D60" s="5"/>
-      <c r="G60" s="5"/>
       <c r="H60" s="5"/>
-      <c r="I60" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I60" s="5"/>
       <c r="J60" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="K60" s="5"/>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K60" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="L60" s="5"/>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D61" s="5"/>
-      <c r="G61" s="5"/>
       <c r="H61" s="5"/>
-      <c r="I61" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I61" s="5"/>
       <c r="J61" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="K61" s="5"/>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K61" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="L61" s="5"/>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="D62" s="5"/>
-      <c r="G62" s="5"/>
+        <v>186</v>
+      </c>
+      <c r="C62" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>287</v>
+      </c>
       <c r="H62" s="5"/>
-      <c r="I62" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I62" s="5"/>
       <c r="J62" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="K62" s="5"/>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K62" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="L62" s="5"/>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D63" s="5"/>
-      <c r="G63" s="5"/>
       <c r="H63" s="5"/>
-      <c r="I63" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I63" s="5"/>
       <c r="J63" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="K63" s="5"/>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K63" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="L63" s="5"/>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B64" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="D64" s="5"/>
+      <c r="H64" s="5"/>
+      <c r="I64" s="5"/>
+      <c r="J64" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K64" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="D64" s="5"/>
-      <c r="G64" s="5"/>
-      <c r="H64" s="5"/>
-      <c r="I64" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J64" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="K64" s="5"/>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L64" s="5"/>
+    </row>
+    <row r="65" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C65" s="5" t="s">
-        <v>307</v>
-      </c>
-      <c r="D65" s="5" t="s">
-        <v>293</v>
-      </c>
-      <c r="E65" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="G65" s="5"/>
+        <v>194</v>
+      </c>
+      <c r="D65" s="5"/>
       <c r="H65" s="5"/>
-      <c r="I65" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I65" s="5"/>
       <c r="J65" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="K65" s="5"/>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K65" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L65" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="D66" s="5"/>
+      <c r="H66" s="5"/>
+      <c r="I66" s="5"/>
+      <c r="J66" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K66" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L66" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="B66" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="D66" s="5"/>
-      <c r="G66" s="5"/>
-      <c r="H66" s="5"/>
-      <c r="I66" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J66" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="K66" s="5"/>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="67" spans="1:12" ht="36" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
         <v>198</v>
       </c>
@@ -3149,17 +3175,19 @@
         <v>199</v>
       </c>
       <c r="D67" s="5"/>
-      <c r="G67" s="5"/>
       <c r="H67" s="5"/>
-      <c r="I67" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I67" s="5"/>
       <c r="J67" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="K67" s="5"/>
-    </row>
-    <row r="68" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="K67" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L67" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
         <v>200</v>
       </c>
@@ -3167,59 +3195,59 @@
         <v>201</v>
       </c>
       <c r="D68" s="5"/>
-      <c r="G68" s="5"/>
       <c r="H68" s="5"/>
-      <c r="I68" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I68" s="5"/>
       <c r="J68" s="5" t="s">
-        <v>83</v>
+        <v>7</v>
       </c>
       <c r="K68" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L68" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A69" s="5" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="69" spans="1:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="A69" s="5" t="s">
+      <c r="B69" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="B69" s="4" t="s">
+      <c r="D69" s="5"/>
+      <c r="H69" s="5"/>
+      <c r="I69" s="5"/>
+      <c r="J69" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K69" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L69" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" ht="36" x14ac:dyDescent="0.3">
+      <c r="A70" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="D69" s="5"/>
-      <c r="G69" s="5"/>
-      <c r="H69" s="5"/>
-      <c r="I69" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J69" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="K69" s="5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" ht="36" x14ac:dyDescent="0.3">
-      <c r="A70" s="5" t="s">
+      <c r="B70" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="B70" s="4" t="s">
+      <c r="D70" s="5"/>
+      <c r="H70" s="5"/>
+      <c r="I70" s="5"/>
+      <c r="J70" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K70" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="D70" s="5"/>
-      <c r="G70" s="5"/>
-      <c r="H70" s="5"/>
-      <c r="I70" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J70" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="K70" s="5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L70" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" ht="36" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
         <v>207</v>
       </c>
@@ -3227,19 +3255,19 @@
         <v>208</v>
       </c>
       <c r="D71" s="5"/>
-      <c r="G71" s="5"/>
       <c r="H71" s="5"/>
-      <c r="I71" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I71" s="5"/>
       <c r="J71" s="5" t="s">
-        <v>83</v>
+        <v>7</v>
       </c>
       <c r="K71" s="5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+        <v>206</v>
+      </c>
+      <c r="L71" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" ht="36" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
         <v>209</v>
       </c>
@@ -3247,19 +3275,19 @@
         <v>210</v>
       </c>
       <c r="D72" s="5"/>
-      <c r="G72" s="5"/>
       <c r="H72" s="5"/>
-      <c r="I72" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I72" s="5"/>
       <c r="J72" s="5" t="s">
-        <v>83</v>
+        <v>7</v>
       </c>
       <c r="K72" s="5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" ht="36" x14ac:dyDescent="0.3">
+        <v>206</v>
+      </c>
+      <c r="L72" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" ht="36" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
         <v>211</v>
       </c>
@@ -3267,119 +3295,119 @@
         <v>212</v>
       </c>
       <c r="D73" s="5"/>
-      <c r="G73" s="5"/>
       <c r="H73" s="5"/>
-      <c r="I73" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I73" s="5"/>
       <c r="J73" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K73" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="L73" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" ht="36" x14ac:dyDescent="0.3">
+      <c r="A74" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="K73" s="5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" ht="36" x14ac:dyDescent="0.3">
-      <c r="A74" s="5" t="s">
+      <c r="B74" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="B74" s="4" t="s">
+      <c r="D74" s="5"/>
+      <c r="H74" s="5"/>
+      <c r="I74" s="5"/>
+      <c r="J74" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K74" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="L74" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A75" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D74" s="5"/>
-      <c r="G74" s="5"/>
-      <c r="H74" s="5"/>
-      <c r="I74" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J74" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="K74" s="5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" ht="36" x14ac:dyDescent="0.3">
-      <c r="A75" s="5" t="s">
+      <c r="B75" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="B75" s="4" t="s">
+      <c r="D75" s="5"/>
+      <c r="H75" s="5"/>
+      <c r="I75" s="5"/>
+      <c r="J75" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K75" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D75" s="5"/>
-      <c r="G75" s="5"/>
-      <c r="H75" s="5"/>
-      <c r="I75" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J75" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="K75" s="5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" ht="36" x14ac:dyDescent="0.3">
+      <c r="L75" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="D76" s="5"/>
+      <c r="H76" s="5"/>
+      <c r="I76" s="5"/>
+      <c r="J76" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K76" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="L76" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="B76" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="D76" s="5"/>
-      <c r="G76" s="5"/>
-      <c r="H76" s="5"/>
-      <c r="I76" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J76" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="K76" s="5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" ht="36" x14ac:dyDescent="0.3">
+    </row>
+    <row r="77" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D77" s="5"/>
-      <c r="G77" s="5"/>
       <c r="H77" s="5"/>
-      <c r="I77" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I77" s="5"/>
       <c r="J77" s="5" t="s">
-        <v>213</v>
+        <v>7</v>
       </c>
       <c r="K77" s="5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+        <v>217</v>
+      </c>
+      <c r="L77" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D78" s="5"/>
-      <c r="G78" s="5"/>
       <c r="H78" s="5"/>
-      <c r="I78" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I78" s="5"/>
       <c r="J78" s="5" t="s">
-        <v>224</v>
+        <v>7</v>
       </c>
       <c r="K78" s="5" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="79" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L78" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" ht="36" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
         <v>226</v>
       </c>
@@ -3387,19 +3415,19 @@
         <v>227</v>
       </c>
       <c r="D79" s="5"/>
-      <c r="G79" s="5"/>
       <c r="H79" s="5"/>
-      <c r="I79" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I79" s="5"/>
       <c r="J79" s="5" t="s">
-        <v>224</v>
+        <v>7</v>
       </c>
       <c r="K79" s="5" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="80" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L79" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
         <v>228</v>
       </c>
@@ -3407,79 +3435,79 @@
         <v>229</v>
       </c>
       <c r="D80" s="5"/>
-      <c r="G80" s="5"/>
       <c r="H80" s="5"/>
-      <c r="I80" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I80" s="5"/>
       <c r="J80" s="5" t="s">
-        <v>224</v>
+        <v>118</v>
       </c>
       <c r="K80" s="5" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+        <v>230</v>
+      </c>
+      <c r="L80" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D81" s="5"/>
-      <c r="G81" s="5"/>
       <c r="H81" s="5"/>
-      <c r="I81" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I81" s="5"/>
       <c r="J81" s="5" t="s">
-        <v>232</v>
+        <v>7</v>
       </c>
       <c r="K81" s="5" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" ht="36" x14ac:dyDescent="0.3">
+        <v>233</v>
+      </c>
+      <c r="L81" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D82" s="5"/>
-      <c r="G82" s="5"/>
       <c r="H82" s="5"/>
-      <c r="I82" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I82" s="5"/>
       <c r="J82" s="5" t="s">
-        <v>232</v>
+        <v>7</v>
       </c>
       <c r="K82" s="5" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+        <v>236</v>
+      </c>
+      <c r="L82" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A83" s="5" t="s">
-        <v>235</v>
+        <v>93</v>
       </c>
       <c r="B83" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="D83" s="5"/>
+      <c r="H83" s="5"/>
+      <c r="I83" s="5"/>
+      <c r="J83" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K83" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="D83" s="5"/>
-      <c r="G83" s="5"/>
-      <c r="H83" s="5"/>
-      <c r="I83" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="J83" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="K83" s="5" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L83" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" ht="36" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
         <v>238</v>
       </c>
@@ -3487,364 +3515,304 @@
         <v>239</v>
       </c>
       <c r="D84" s="5"/>
-      <c r="G84" s="5"/>
       <c r="H84" s="5"/>
-      <c r="I84" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I84" s="5"/>
       <c r="J84" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K84" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="L84" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A85" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="K84" s="5" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="A85" s="5" t="s">
+      <c r="B85" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="B85" s="4" t="s">
+      <c r="D85" s="5"/>
+      <c r="H85" s="5"/>
+      <c r="I85" s="5"/>
+      <c r="J85" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K85" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="L85" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A86" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="D85" s="5"/>
-      <c r="G85" s="5"/>
-      <c r="H85" s="5"/>
-      <c r="I85" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J85" s="5" t="s">
+      <c r="B86" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="K85" s="5" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="A86" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="B86" s="4" t="s">
+      <c r="D86" s="5"/>
+      <c r="H86" s="5"/>
+      <c r="I86" s="5"/>
+      <c r="J86" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K86" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="L86" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A87" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="D86" s="5"/>
-      <c r="G86" s="5"/>
-      <c r="H86" s="5"/>
-      <c r="I86" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J86" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="K86" s="5" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" ht="36" x14ac:dyDescent="0.3">
-      <c r="A87" s="5" t="s">
+      <c r="B87" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="B87" s="4" t="s">
+      <c r="D87" s="5"/>
+      <c r="H87" s="5"/>
+      <c r="I87" s="5"/>
+      <c r="J87" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K87" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="L87" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A88" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="D87" s="5"/>
-      <c r="G87" s="5"/>
-      <c r="H87" s="5"/>
-      <c r="I87" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J87" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="K87" s="5" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="A88" s="5" t="s">
+      <c r="B88" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="B88" s="4" t="s">
+      <c r="D88" s="5"/>
+      <c r="H88" s="5"/>
+      <c r="I88" s="5"/>
+      <c r="J88" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K88" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="L88" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A89" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="D88" s="5"/>
-      <c r="G88" s="5"/>
-      <c r="H88" s="5"/>
-      <c r="I88" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J88" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="K88" s="5" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="89" spans="1:11" ht="24" x14ac:dyDescent="0.3">
-      <c r="A89" s="5" t="s">
+      <c r="B89" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="B89" s="4" t="s">
+      <c r="D89" s="5"/>
+      <c r="H89" s="5"/>
+      <c r="I89" s="5"/>
+      <c r="J89" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K89" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="D89" s="5"/>
-      <c r="G89" s="5"/>
-      <c r="H89" s="5"/>
-      <c r="I89" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J89" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="K89" s="5" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="90" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="L89" s="5" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A90" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="D90" s="5"/>
+      <c r="H90" s="5"/>
+      <c r="I90" s="5"/>
+      <c r="J90" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K90" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="L90" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="B90" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="D90" s="5"/>
-      <c r="G90" s="5"/>
-      <c r="H90" s="5"/>
-      <c r="I90" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J90" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="K90" s="5" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="91" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+    </row>
+    <row r="91" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D91" s="5"/>
-      <c r="G91" s="5"/>
       <c r="H91" s="5"/>
-      <c r="I91" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I91" s="5"/>
       <c r="J91" s="5" t="s">
-        <v>243</v>
+        <v>7</v>
       </c>
       <c r="K91" s="5" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+        <v>256</v>
+      </c>
+      <c r="L91" s="5" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A92" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D92" s="5"/>
-      <c r="G92" s="5"/>
       <c r="H92" s="5"/>
-      <c r="I92" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I92" s="5"/>
       <c r="J92" s="5" t="s">
-        <v>257</v>
+        <v>7</v>
       </c>
       <c r="K92" s="5" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+        <v>259</v>
+      </c>
+      <c r="L92" s="5" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B93" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D93" s="5"/>
+      <c r="H93" s="5"/>
+      <c r="I93" s="5"/>
+      <c r="J93" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K93" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="L93" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="D93" s="5"/>
-      <c r="G93" s="5"/>
-      <c r="H93" s="5"/>
-      <c r="I93" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J93" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="K93" s="5" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="94" spans="1:11" ht="24" x14ac:dyDescent="0.3">
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A94" s="5" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D94" s="5"/>
-      <c r="G94" s="5"/>
       <c r="H94" s="5"/>
-      <c r="I94" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I94" s="5"/>
       <c r="J94" s="5" t="s">
-        <v>263</v>
+        <v>7</v>
       </c>
       <c r="K94" s="5" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+        <v>266</v>
+      </c>
+      <c r="L94" s="5" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="D95" s="5"/>
-      <c r="G95" s="5"/>
       <c r="H95" s="5"/>
-      <c r="I95" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I95" s="5"/>
       <c r="J95" s="5" t="s">
-        <v>266</v>
+        <v>7</v>
       </c>
       <c r="K95" s="5" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
+        <v>269</v>
+      </c>
+      <c r="L95" s="5" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A96" s="5" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D96" s="5"/>
-      <c r="G96" s="5"/>
       <c r="H96" s="5"/>
-      <c r="I96" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I96" s="5"/>
       <c r="J96" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K96" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="L96" s="5" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A97" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="D97" s="5"/>
+      <c r="H97" s="5"/>
+      <c r="I97" s="5"/>
+      <c r="J97" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K97" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="L97" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="K96" s="5" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A97" s="5" t="s">
-        <v>271</v>
-      </c>
-      <c r="B97" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="D97" s="5"/>
-      <c r="G97" s="5"/>
-      <c r="H97" s="5"/>
-      <c r="I97" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J97" s="5" t="s">
-        <v>273</v>
-      </c>
-      <c r="K97" s="5" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="98" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="D98" s="5"/>
-      <c r="G98" s="5"/>
       <c r="H98" s="5"/>
-      <c r="I98" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="I98" s="5"/>
       <c r="J98" s="5" t="s">
-        <v>276</v>
+        <v>7</v>
       </c>
       <c r="K98" s="5" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A99" s="5" t="s">
-        <v>278</v>
-      </c>
-      <c r="B99" s="4" t="s">
-        <v>279</v>
-      </c>
-      <c r="D99" s="5"/>
-      <c r="G99" s="5"/>
-      <c r="H99" s="5"/>
-      <c r="I99" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J99" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="K99" s="5" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A100" s="5" t="s">
-        <v>282</v>
-      </c>
-      <c r="B100" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="D100" s="5"/>
-      <c r="G100" s="5"/>
-      <c r="H100" s="5"/>
-      <c r="I100" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J100" s="5" t="s">
-        <v>284</v>
-      </c>
-      <c r="K100" s="5" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A101" s="5" t="s">
-        <v>285</v>
-      </c>
-      <c r="B101" s="4" t="s">
-        <v>286</v>
-      </c>
-      <c r="D101" s="5"/>
-      <c r="G101" s="5"/>
-      <c r="H101" s="5"/>
-      <c r="I101" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J101" s="5" t="s">
-        <v>287</v>
-      </c>
-      <c r="K101" s="5" t="s">
-        <v>277</v>
+      <c r="L98" s="5" t="s">
+        <v>270</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F1:F1048576 D1:D1048576">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="No">
+  <conditionalFormatting sqref="F1:G1048576 D1:D1048576">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH("No",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Yes">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Yes">
       <formula>NOT(ISERROR(SEARCH("Yes",D1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Update intent test cases spreadsheet
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Cidy_Intent_Test_Cases_90.xlsx
+++ b/documentation/Cidy_Intent_Test_Cases_90.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RRAPOPOR\Documents\Cidy testing\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB8AC034-0F9F-47FC-AF32-615409B689EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B682ABC-EC51-4A9D-88FF-BE0B9D22B4C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="2" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="381">
   <si>
     <t>Scenario</t>
   </si>
@@ -1941,7 +1941,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1969,6 +1969,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2001,7 +2025,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2026,8 +2050,6 @@
     </xf>
     <xf numFmtId="9" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -2041,6 +2063,11 @@
     <xf numFmtId="9" fontId="4" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="9" fontId="4" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="9" fontId="4" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="9" fontId="4" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="9" fontId="4" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2823,19 +2850,19 @@
       <c r="H4" s="10" t="s">
         <v>370</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="J4" s="24" t="s">
         <v>379</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="K4" s="25" t="s">
         <v>380</v>
       </c>
-      <c r="L4" s="12" t="s">
+      <c r="L4" s="26" t="s">
         <v>193</v>
       </c>
-      <c r="M4" s="13" t="s">
+      <c r="M4" s="27" t="s">
         <v>263</v>
       </c>
       <c r="O4" s="13"/>
@@ -2858,12 +2885,14 @@
         <v>0.53846153846153844</v>
       </c>
       <c r="E5" s="11"/>
-      <c r="G5" s="13" t="str" cm="1">
+      <c r="G5" s="16" t="str" cm="1">
         <f t="array" ref="G5:G15">_xlfn._xlws.SORT(_xlfn.UNIQUE(_xlfn._xlws.FILTER('Test Cases'!B2:B1000,'Test Cases'!B2:B1000&lt;&gt;"")))</f>
         <v>About Cidy</v>
       </c>
-      <c r="H5" s="13"/>
-      <c r="I5" s="14" cm="1">
+      <c r="H5" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="I5" s="17" cm="1">
         <f t="array" ref="I5:I15">_xlfn.MAP(_xlfn.ANCHORARRAY(G5),_xlfn.LAMBDA(_xlpm.topic,
   _xlfn.LET(
     _xlpm.topics,'Test Cases'!B2:B1000,
@@ -2874,7 +2903,7 @@
 ))</f>
         <v>0.18181818181818182</v>
       </c>
-      <c r="J5" s="14" cm="1">
+      <c r="J5" s="17" cm="1">
         <f t="array" ref="J5:J15">_xlfn.MAP(_xlfn.ANCHORARRAY(G5),_xlfn.LAMBDA(_xlpm.topic,
   _xlfn.LET(
     _xlpm.topics,'Test Cases'!B2:B1000,
@@ -2885,7 +2914,7 @@
 ))</f>
         <v>0.18181818181818182</v>
       </c>
-      <c r="K5" s="14" t="str" cm="1">
+      <c r="K5" s="17" t="str" cm="1">
         <f t="array" ref="K5:K15">_xlfn.MAP(_xlfn.ANCHORARRAY(G5),_xlfn.LAMBDA(_xlpm.topic,
   _xlfn.LET(
     _xlpm.scores,_xlfn._xlws.FILTER(
@@ -2899,7 +2928,7 @@
 ))</f>
         <v>NA</v>
       </c>
-      <c r="L5" s="14" cm="1">
+      <c r="L5" s="17" cm="1">
         <f t="array" ref="L5:L15">_xlfn.MAP(_xlfn.ANCHORARRAY(G5),_xlfn.LAMBDA(_xlpm.topic,
   _xlfn.LET(
     _xlpm.topics,'Test Cases'!B2:B1000,
@@ -2910,7 +2939,7 @@
 ))</f>
         <v>0.45454545454545453</v>
       </c>
-      <c r="M5" s="15" cm="1">
+      <c r="M5" s="18" cm="1">
         <f t="array" ref="M5:M15">_xlfn.MAP(_xlfn.ANCHORARRAY(G5),_xlfn.LAMBDA(_xlpm.topic,
   _xlfn.LET(
     _xlpm.topics,'Test Cases'!B2:B1000,
@@ -2929,7 +2958,7 @@
 )</f>
         <v>Clarification path</v>
       </c>
-      <c r="P5" s="16" cm="1">
+      <c r="P5" s="14" cm="1">
         <f t="array" ref="P5:P12">_xlfn.MAP(_xlfn.ANCHORARRAY(O5),_xlfn.LAMBDA(_xlpm.path,
   _xlfn.LET(
     _xlpm.src,_xlfn._xlws.FILTER('Test Cases'!A2:F1000,ISNUMBER(SEARCH("-",'Test Cases'!A2:A1000))),
@@ -2941,7 +2970,7 @@
 ))</f>
         <v>5.2631578947368418E-2</v>
       </c>
-      <c r="Q5" s="16" cm="1">
+      <c r="Q5" s="14" cm="1">
         <f t="array" ref="Q5:Q12">_xlfn.MAP(_xlfn.ANCHORARRAY(O5),_xlfn.LAMBDA(_xlpm.path,
   _xlfn.LET(
     _xlpm.src,_xlfn._xlws.FILTER('Test Cases'!A2:F1000,ISNUMBER(SEARCH("-",'Test Cases'!A2:A1000))),
@@ -2953,7 +2982,7 @@
 ))</f>
         <v>5.2631578947368418E-2</v>
       </c>
-      <c r="R5" s="16" cm="1">
+      <c r="R5" s="14" cm="1">
         <f t="array" ref="R5:R12">_xlfn.MAP(_xlfn.ANCHORARRAY(O5),_xlfn.LAMBDA(_xlpm.path,
   _xlfn.LET(
     _xlpm.src,_xlfn._xlws.FILTER('Test Cases'!A2:F1000,ISNUMBER(SEARCH("-",'Test Cases'!A2:A1000))),
@@ -2970,84 +2999,84 @@
       <c r="C6" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="D6" s="17">
+      <c r="D6" s="15">
         <f>COUNTBLANK('Test Cases'!F2:F101)/ROWS('Test Cases'!F2:F101)</f>
         <v>0.36</v>
       </c>
       <c r="E6" s="11"/>
-      <c r="G6" s="18" t="str">
+      <c r="G6" s="16" t="str">
         <v>Country Data</v>
       </c>
-      <c r="H6" s="18" t="s">
+      <c r="H6" s="16" t="s">
         <v>367</v>
       </c>
-      <c r="I6" s="19">
+      <c r="I6" s="17">
         <v>1</v>
       </c>
-      <c r="J6" s="19">
+      <c r="J6" s="17">
         <v>0.5</v>
       </c>
-      <c r="K6" s="24">
+      <c r="K6" s="22">
         <v>2.75</v>
       </c>
-      <c r="L6" s="19">
+      <c r="L6" s="17">
         <v>0</v>
       </c>
-      <c r="M6" s="20">
+      <c r="M6" s="18">
         <v>0</v>
       </c>
       <c r="O6" s="13" t="str">
         <v>Exit Cidy flow command</v>
       </c>
-      <c r="P6" s="16">
+      <c r="P6" s="14">
         <v>0</v>
       </c>
-      <c r="Q6" s="16">
+      <c r="Q6" s="14">
         <v>0</v>
       </c>
-      <c r="R6" s="16">
+      <c r="R6" s="14">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="G7" s="18" t="str">
+      <c r="G7" s="16" t="str">
         <v>DA</v>
       </c>
-      <c r="H7" s="18" t="s">
-        <v>368</v>
-      </c>
-      <c r="I7" s="19">
+      <c r="H7" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="I7" s="17">
         <v>0.81818181818181823</v>
       </c>
-      <c r="J7" s="19">
+      <c r="J7" s="17">
         <v>0.72727272727272729</v>
       </c>
-      <c r="K7" s="19" t="str">
+      <c r="K7" s="17" t="str">
         <v>NA</v>
       </c>
-      <c r="L7" s="19">
+      <c r="L7" s="17">
         <v>0.18181818181818182</v>
       </c>
-      <c r="M7" s="20">
+      <c r="M7" s="18">
         <v>0</v>
       </c>
       <c r="O7" s="13" t="str">
         <v>Greeting guard</v>
       </c>
-      <c r="P7" s="16">
+      <c r="P7" s="14">
         <v>1</v>
       </c>
-      <c r="Q7" s="16">
+      <c r="Q7" s="14">
         <v>0</v>
       </c>
-      <c r="R7" s="16">
+      <c r="R7" s="14">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="C8" s="21"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="21"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
       <c r="G8" s="13" t="str">
         <v>Evaluation</v>
       </c>
@@ -3064,19 +3093,19 @@
       <c r="L8" s="12">
         <v>0.7142857142857143</v>
       </c>
-      <c r="M8" s="16">
+      <c r="M8" s="14">
         <v>0.14285714285714285</v>
       </c>
       <c r="O8" s="13" t="str">
         <v>Greeting path</v>
       </c>
-      <c r="P8" s="16">
+      <c r="P8" s="14">
         <v>0</v>
       </c>
-      <c r="Q8" s="16">
+      <c r="Q8" s="14">
         <v>0</v>
       </c>
-      <c r="R8" s="16">
+      <c r="R8" s="14">
         <v>1</v>
       </c>
     </row>
@@ -3097,19 +3126,19 @@
       <c r="L9" s="12">
         <v>0</v>
       </c>
-      <c r="M9" s="16">
+      <c r="M9" s="14">
         <v>1</v>
       </c>
-      <c r="O9" s="18" t="str">
+      <c r="O9" s="16" t="str">
         <v>Happy path</v>
       </c>
-      <c r="P9" s="20">
+      <c r="P9" s="18">
         <v>0.31746031746031744</v>
       </c>
-      <c r="Q9" s="20">
+      <c r="Q9" s="18">
         <v>0.52380952380952384</v>
       </c>
-      <c r="R9" s="20">
+      <c r="R9" s="18">
         <v>0.15873015873015872</v>
       </c>
     </row>
@@ -3130,19 +3159,19 @@
       <c r="L10" s="12">
         <v>0</v>
       </c>
-      <c r="M10" s="16">
+      <c r="M10" s="14">
         <v>0.66666666666666663</v>
       </c>
       <c r="O10" s="13" t="str">
         <v>Out of scope</v>
       </c>
-      <c r="P10" s="16">
+      <c r="P10" s="14">
         <v>1</v>
       </c>
-      <c r="Q10" s="16">
+      <c r="Q10" s="14">
         <v>0</v>
       </c>
-      <c r="R10" s="16">
+      <c r="R10" s="14">
         <v>0</v>
       </c>
     </row>
@@ -3163,19 +3192,19 @@
       <c r="L11" s="12">
         <v>4.7619047619047616E-2</v>
       </c>
-      <c r="M11" s="16">
+      <c r="M11" s="14">
         <v>0.90476190476190477</v>
       </c>
       <c r="O11" s="13" t="str">
         <v>Regression</v>
       </c>
-      <c r="P11" s="16">
+      <c r="P11" s="14">
         <v>1</v>
       </c>
-      <c r="Q11" s="16">
+      <c r="Q11" s="14">
         <v>0</v>
       </c>
-      <c r="R11" s="16">
+      <c r="R11" s="14">
         <v>0</v>
       </c>
     </row>
@@ -3196,42 +3225,42 @@
       <c r="L12" s="12">
         <v>0</v>
       </c>
-      <c r="M12" s="16">
+      <c r="M12" s="14">
         <v>0</v>
       </c>
       <c r="O12" s="13" t="str">
         <v>Vague path</v>
       </c>
-      <c r="P12" s="16">
+      <c r="P12" s="14">
         <v>0.2</v>
       </c>
-      <c r="Q12" s="16">
+      <c r="Q12" s="14">
         <v>0.2</v>
       </c>
-      <c r="R12" s="16">
+      <c r="R12" s="14">
         <v>0.6</v>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="G13" s="18" t="str">
+      <c r="G13" s="16" t="str">
         <v>PD</v>
       </c>
-      <c r="H13" s="18" t="s">
-        <v>369</v>
-      </c>
-      <c r="I13" s="19">
+      <c r="H13" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="I13" s="17">
         <v>0.2857142857142857</v>
       </c>
-      <c r="J13" s="19">
+      <c r="J13" s="17">
         <v>0.2857142857142857</v>
       </c>
-      <c r="K13" s="19" t="str">
+      <c r="K13" s="17" t="str">
         <v>NA</v>
       </c>
-      <c r="L13" s="19">
+      <c r="L13" s="17">
         <v>0.6428571428571429</v>
       </c>
-      <c r="M13" s="20">
+      <c r="M13" s="18">
         <v>7.1428571428571425E-2</v>
       </c>
     </row>
@@ -3252,369 +3281,371 @@
       <c r="L14" s="12">
         <v>0.5</v>
       </c>
-      <c r="M14" s="16">
+      <c r="M14" s="14">
         <v>0.5</v>
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="G15" s="13" t="str">
+      <c r="G15" s="16" t="str">
         <v>RPTC</v>
       </c>
-      <c r="H15" s="13"/>
-      <c r="I15" s="12">
+      <c r="H15" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="I15" s="17">
         <v>0.1111111111111111</v>
       </c>
-      <c r="J15" s="12">
+      <c r="J15" s="17">
         <v>0.1111111111111111</v>
       </c>
-      <c r="K15" s="12" t="str">
+      <c r="K15" s="17" t="str">
         <v>NA</v>
       </c>
-      <c r="L15" s="12">
+      <c r="L15" s="17">
         <v>0.66666666666666663</v>
       </c>
-      <c r="M15" s="16">
+      <c r="M15" s="18">
         <v>0.22222222222222221</v>
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="I16" s="22"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
-      <c r="L16" s="22"/>
-      <c r="M16" s="23"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="20"/>
+      <c r="L16" s="20"/>
+      <c r="M16" s="21"/>
     </row>
     <row r="17" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I17" s="22"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="22"/>
-      <c r="L17" s="22"/>
-      <c r="M17" s="23"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
+      <c r="L17" s="20"/>
+      <c r="M17" s="21"/>
     </row>
     <row r="18" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="22"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="23"/>
+      <c r="I18" s="20"/>
+      <c r="J18" s="20"/>
+      <c r="K18" s="20"/>
+      <c r="L18" s="20"/>
+      <c r="M18" s="21"/>
     </row>
     <row r="19" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I19" s="22"/>
-      <c r="J19" s="22"/>
-      <c r="K19" s="22"/>
-      <c r="L19" s="22"/>
-      <c r="M19" s="23"/>
+      <c r="I19" s="20"/>
+      <c r="J19" s="20"/>
+      <c r="K19" s="20"/>
+      <c r="L19" s="20"/>
+      <c r="M19" s="21"/>
     </row>
     <row r="20" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I20" s="22"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="22"/>
-      <c r="L20" s="22"/>
-      <c r="M20" s="23"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="20"/>
+      <c r="K20" s="20"/>
+      <c r="L20" s="20"/>
+      <c r="M20" s="21"/>
     </row>
     <row r="21" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I21" s="22"/>
-      <c r="J21" s="22"/>
-      <c r="K21" s="22"/>
-      <c r="L21" s="22"/>
-      <c r="M21" s="23"/>
+      <c r="I21" s="20"/>
+      <c r="J21" s="20"/>
+      <c r="K21" s="20"/>
+      <c r="L21" s="20"/>
+      <c r="M21" s="21"/>
     </row>
     <row r="22" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I22" s="22"/>
-      <c r="J22" s="22"/>
-      <c r="K22" s="22"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="23"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
+      <c r="L22" s="20"/>
+      <c r="M22" s="21"/>
     </row>
     <row r="23" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I23" s="22"/>
-      <c r="J23" s="22"/>
-      <c r="K23" s="22"/>
-      <c r="L23" s="22"/>
-      <c r="M23" s="23"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="20"/>
+      <c r="K23" s="20"/>
+      <c r="L23" s="20"/>
+      <c r="M23" s="21"/>
     </row>
     <row r="24" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I24" s="22"/>
-      <c r="J24" s="22"/>
-      <c r="K24" s="22"/>
-      <c r="L24" s="22"/>
-      <c r="M24" s="23"/>
+      <c r="I24" s="20"/>
+      <c r="J24" s="20"/>
+      <c r="K24" s="20"/>
+      <c r="L24" s="20"/>
+      <c r="M24" s="21"/>
     </row>
     <row r="25" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I25" s="22"/>
-      <c r="J25" s="22"/>
-      <c r="K25" s="22"/>
-      <c r="L25" s="22"/>
-      <c r="M25" s="23"/>
+      <c r="I25" s="20"/>
+      <c r="J25" s="20"/>
+      <c r="K25" s="20"/>
+      <c r="L25" s="20"/>
+      <c r="M25" s="21"/>
     </row>
     <row r="26" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I26" s="22"/>
-      <c r="J26" s="22"/>
-      <c r="K26" s="22"/>
-      <c r="L26" s="22"/>
-      <c r="M26" s="23"/>
+      <c r="I26" s="20"/>
+      <c r="J26" s="20"/>
+      <c r="K26" s="20"/>
+      <c r="L26" s="20"/>
+      <c r="M26" s="21"/>
     </row>
     <row r="27" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I27" s="22"/>
-      <c r="J27" s="22"/>
-      <c r="K27" s="22"/>
-      <c r="L27" s="22"/>
-      <c r="M27" s="23"/>
+      <c r="I27" s="20"/>
+      <c r="J27" s="20"/>
+      <c r="K27" s="20"/>
+      <c r="L27" s="20"/>
+      <c r="M27" s="21"/>
     </row>
     <row r="28" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I28" s="22"/>
-      <c r="J28" s="22"/>
-      <c r="K28" s="22"/>
-      <c r="L28" s="22"/>
-      <c r="M28" s="23"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="20"/>
+      <c r="K28" s="20"/>
+      <c r="L28" s="20"/>
+      <c r="M28" s="21"/>
     </row>
     <row r="29" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I29" s="22"/>
-      <c r="J29" s="22"/>
-      <c r="K29" s="22"/>
-      <c r="L29" s="22"/>
-      <c r="M29" s="23"/>
+      <c r="I29" s="20"/>
+      <c r="J29" s="20"/>
+      <c r="K29" s="20"/>
+      <c r="L29" s="20"/>
+      <c r="M29" s="21"/>
     </row>
     <row r="30" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I30" s="22"/>
-      <c r="J30" s="22"/>
-      <c r="K30" s="22"/>
-      <c r="L30" s="22"/>
-      <c r="M30" s="23"/>
+      <c r="I30" s="20"/>
+      <c r="J30" s="20"/>
+      <c r="K30" s="20"/>
+      <c r="L30" s="20"/>
+      <c r="M30" s="21"/>
     </row>
     <row r="31" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I31" s="22"/>
-      <c r="J31" s="22"/>
-      <c r="K31" s="22"/>
-      <c r="L31" s="22"/>
-      <c r="M31" s="23"/>
+      <c r="I31" s="20"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="20"/>
+      <c r="L31" s="20"/>
+      <c r="M31" s="21"/>
     </row>
     <row r="32" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I32" s="22"/>
-      <c r="J32" s="22"/>
-      <c r="K32" s="22"/>
-      <c r="L32" s="22"/>
-      <c r="M32" s="23"/>
+      <c r="I32" s="20"/>
+      <c r="J32" s="20"/>
+      <c r="K32" s="20"/>
+      <c r="L32" s="20"/>
+      <c r="M32" s="21"/>
     </row>
     <row r="33" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I33" s="22"/>
-      <c r="J33" s="22"/>
-      <c r="K33" s="22"/>
-      <c r="L33" s="22"/>
-      <c r="M33" s="23"/>
+      <c r="I33" s="20"/>
+      <c r="J33" s="20"/>
+      <c r="K33" s="20"/>
+      <c r="L33" s="20"/>
+      <c r="M33" s="21"/>
     </row>
     <row r="34" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I34" s="22"/>
-      <c r="J34" s="22"/>
-      <c r="K34" s="22"/>
-      <c r="L34" s="22"/>
-      <c r="M34" s="23"/>
+      <c r="I34" s="20"/>
+      <c r="J34" s="20"/>
+      <c r="K34" s="20"/>
+      <c r="L34" s="20"/>
+      <c r="M34" s="21"/>
     </row>
     <row r="35" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I35" s="22"/>
-      <c r="J35" s="22"/>
-      <c r="K35" s="22"/>
-      <c r="L35" s="22"/>
-      <c r="M35" s="23"/>
+      <c r="I35" s="20"/>
+      <c r="J35" s="20"/>
+      <c r="K35" s="20"/>
+      <c r="L35" s="20"/>
+      <c r="M35" s="21"/>
     </row>
     <row r="36" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I36" s="22"/>
-      <c r="J36" s="22"/>
-      <c r="K36" s="22"/>
-      <c r="L36" s="22"/>
-      <c r="M36" s="23"/>
+      <c r="I36" s="20"/>
+      <c r="J36" s="20"/>
+      <c r="K36" s="20"/>
+      <c r="L36" s="20"/>
+      <c r="M36" s="21"/>
     </row>
     <row r="37" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I37" s="22"/>
-      <c r="J37" s="22"/>
-      <c r="K37" s="22"/>
-      <c r="L37" s="22"/>
-      <c r="M37" s="23"/>
+      <c r="I37" s="20"/>
+      <c r="J37" s="20"/>
+      <c r="K37" s="20"/>
+      <c r="L37" s="20"/>
+      <c r="M37" s="21"/>
     </row>
     <row r="38" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I38" s="22"/>
-      <c r="J38" s="22"/>
-      <c r="K38" s="22"/>
-      <c r="L38" s="22"/>
-      <c r="M38" s="23"/>
+      <c r="I38" s="20"/>
+      <c r="J38" s="20"/>
+      <c r="K38" s="20"/>
+      <c r="L38" s="20"/>
+      <c r="M38" s="21"/>
     </row>
     <row r="39" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I39" s="22"/>
-      <c r="J39" s="22"/>
-      <c r="K39" s="22"/>
-      <c r="L39" s="22"/>
-      <c r="M39" s="23"/>
+      <c r="I39" s="20"/>
+      <c r="J39" s="20"/>
+      <c r="K39" s="20"/>
+      <c r="L39" s="20"/>
+      <c r="M39" s="21"/>
     </row>
     <row r="40" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I40" s="22"/>
-      <c r="J40" s="22"/>
-      <c r="K40" s="22"/>
-      <c r="L40" s="22"/>
-      <c r="M40" s="23"/>
+      <c r="I40" s="20"/>
+      <c r="J40" s="20"/>
+      <c r="K40" s="20"/>
+      <c r="L40" s="20"/>
+      <c r="M40" s="21"/>
     </row>
     <row r="41" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
-      <c r="K41" s="22"/>
-      <c r="L41" s="22"/>
-      <c r="M41" s="23"/>
+      <c r="I41" s="20"/>
+      <c r="J41" s="20"/>
+      <c r="K41" s="20"/>
+      <c r="L41" s="20"/>
+      <c r="M41" s="21"/>
     </row>
     <row r="42" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I42" s="22"/>
-      <c r="J42" s="22"/>
-      <c r="K42" s="22"/>
-      <c r="L42" s="22"/>
-      <c r="M42" s="23"/>
+      <c r="I42" s="20"/>
+      <c r="J42" s="20"/>
+      <c r="K42" s="20"/>
+      <c r="L42" s="20"/>
+      <c r="M42" s="21"/>
     </row>
     <row r="43" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I43" s="22"/>
-      <c r="J43" s="22"/>
-      <c r="K43" s="22"/>
-      <c r="L43" s="22"/>
-      <c r="M43" s="23"/>
+      <c r="I43" s="20"/>
+      <c r="J43" s="20"/>
+      <c r="K43" s="20"/>
+      <c r="L43" s="20"/>
+      <c r="M43" s="21"/>
     </row>
     <row r="44" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I44" s="22"/>
-      <c r="J44" s="22"/>
-      <c r="K44" s="22"/>
-      <c r="L44" s="22"/>
-      <c r="M44" s="23"/>
+      <c r="I44" s="20"/>
+      <c r="J44" s="20"/>
+      <c r="K44" s="20"/>
+      <c r="L44" s="20"/>
+      <c r="M44" s="21"/>
     </row>
     <row r="45" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I45" s="22"/>
-      <c r="J45" s="22"/>
-      <c r="K45" s="22"/>
-      <c r="L45" s="22"/>
-      <c r="M45" s="23"/>
+      <c r="I45" s="20"/>
+      <c r="J45" s="20"/>
+      <c r="K45" s="20"/>
+      <c r="L45" s="20"/>
+      <c r="M45" s="21"/>
     </row>
     <row r="46" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I46" s="22"/>
-      <c r="J46" s="22"/>
-      <c r="K46" s="22"/>
-      <c r="L46" s="22"/>
-      <c r="M46" s="23"/>
+      <c r="I46" s="20"/>
+      <c r="J46" s="20"/>
+      <c r="K46" s="20"/>
+      <c r="L46" s="20"/>
+      <c r="M46" s="21"/>
     </row>
     <row r="47" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I47" s="22"/>
-      <c r="J47" s="22"/>
-      <c r="K47" s="22"/>
-      <c r="L47" s="22"/>
-      <c r="M47" s="23"/>
+      <c r="I47" s="20"/>
+      <c r="J47" s="20"/>
+      <c r="K47" s="20"/>
+      <c r="L47" s="20"/>
+      <c r="M47" s="21"/>
     </row>
     <row r="48" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I48" s="22"/>
-      <c r="J48" s="22"/>
-      <c r="K48" s="22"/>
-      <c r="L48" s="22"/>
-      <c r="M48" s="23"/>
+      <c r="I48" s="20"/>
+      <c r="J48" s="20"/>
+      <c r="K48" s="20"/>
+      <c r="L48" s="20"/>
+      <c r="M48" s="21"/>
     </row>
     <row r="49" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I49" s="22"/>
-      <c r="J49" s="22"/>
-      <c r="K49" s="22"/>
-      <c r="L49" s="22"/>
-      <c r="M49" s="23"/>
+      <c r="I49" s="20"/>
+      <c r="J49" s="20"/>
+      <c r="K49" s="20"/>
+      <c r="L49" s="20"/>
+      <c r="M49" s="21"/>
     </row>
     <row r="50" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I50" s="22"/>
-      <c r="J50" s="22"/>
-      <c r="K50" s="22"/>
-      <c r="L50" s="22"/>
-      <c r="M50" s="23"/>
+      <c r="I50" s="20"/>
+      <c r="J50" s="20"/>
+      <c r="K50" s="20"/>
+      <c r="L50" s="20"/>
+      <c r="M50" s="21"/>
     </row>
     <row r="51" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I51" s="22"/>
-      <c r="J51" s="22"/>
-      <c r="K51" s="22"/>
-      <c r="L51" s="22"/>
-      <c r="M51" s="23"/>
+      <c r="I51" s="20"/>
+      <c r="J51" s="20"/>
+      <c r="K51" s="20"/>
+      <c r="L51" s="20"/>
+      <c r="M51" s="21"/>
     </row>
     <row r="52" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I52" s="22"/>
-      <c r="J52" s="22"/>
-      <c r="K52" s="22"/>
-      <c r="L52" s="22"/>
-      <c r="M52" s="23"/>
+      <c r="I52" s="20"/>
+      <c r="J52" s="20"/>
+      <c r="K52" s="20"/>
+      <c r="L52" s="20"/>
+      <c r="M52" s="21"/>
     </row>
     <row r="53" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I53" s="22"/>
-      <c r="J53" s="22"/>
-      <c r="K53" s="22"/>
-      <c r="L53" s="22"/>
-      <c r="M53" s="23"/>
+      <c r="I53" s="20"/>
+      <c r="J53" s="20"/>
+      <c r="K53" s="20"/>
+      <c r="L53" s="20"/>
+      <c r="M53" s="21"/>
     </row>
     <row r="54" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I54" s="22"/>
-      <c r="J54" s="22"/>
-      <c r="K54" s="22"/>
-      <c r="L54" s="22"/>
-      <c r="M54" s="23"/>
+      <c r="I54" s="20"/>
+      <c r="J54" s="20"/>
+      <c r="K54" s="20"/>
+      <c r="L54" s="20"/>
+      <c r="M54" s="21"/>
     </row>
     <row r="55" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I55" s="22"/>
-      <c r="J55" s="22"/>
-      <c r="K55" s="22"/>
-      <c r="L55" s="22"/>
-      <c r="M55" s="23"/>
+      <c r="I55" s="20"/>
+      <c r="J55" s="20"/>
+      <c r="K55" s="20"/>
+      <c r="L55" s="20"/>
+      <c r="M55" s="21"/>
     </row>
     <row r="56" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I56" s="22"/>
-      <c r="J56" s="22"/>
-      <c r="K56" s="22"/>
-      <c r="L56" s="22"/>
-      <c r="M56" s="23"/>
+      <c r="I56" s="20"/>
+      <c r="J56" s="20"/>
+      <c r="K56" s="20"/>
+      <c r="L56" s="20"/>
+      <c r="M56" s="21"/>
     </row>
     <row r="57" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I57" s="22"/>
-      <c r="J57" s="22"/>
-      <c r="K57" s="22"/>
-      <c r="L57" s="22"/>
-      <c r="M57" s="23"/>
+      <c r="I57" s="20"/>
+      <c r="J57" s="20"/>
+      <c r="K57" s="20"/>
+      <c r="L57" s="20"/>
+      <c r="M57" s="21"/>
     </row>
     <row r="58" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I58" s="22"/>
-      <c r="J58" s="22"/>
-      <c r="K58" s="22"/>
-      <c r="L58" s="22"/>
-      <c r="M58" s="23"/>
+      <c r="I58" s="20"/>
+      <c r="J58" s="20"/>
+      <c r="K58" s="20"/>
+      <c r="L58" s="20"/>
+      <c r="M58" s="21"/>
     </row>
     <row r="59" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I59" s="22"/>
-      <c r="J59" s="22"/>
-      <c r="K59" s="22"/>
-      <c r="L59" s="22"/>
-      <c r="M59" s="23"/>
+      <c r="I59" s="20"/>
+      <c r="J59" s="20"/>
+      <c r="K59" s="20"/>
+      <c r="L59" s="20"/>
+      <c r="M59" s="21"/>
     </row>
     <row r="60" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I60" s="22"/>
-      <c r="J60" s="22"/>
-      <c r="K60" s="22"/>
-      <c r="L60" s="22"/>
-      <c r="M60" s="23"/>
+      <c r="I60" s="20"/>
+      <c r="J60" s="20"/>
+      <c r="K60" s="20"/>
+      <c r="L60" s="20"/>
+      <c r="M60" s="21"/>
     </row>
     <row r="61" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I61" s="22"/>
-      <c r="J61" s="22"/>
-      <c r="K61" s="22"/>
-      <c r="L61" s="22"/>
-      <c r="M61" s="23"/>
+      <c r="I61" s="20"/>
+      <c r="J61" s="20"/>
+      <c r="K61" s="20"/>
+      <c r="L61" s="20"/>
+      <c r="M61" s="21"/>
     </row>
     <row r="62" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I62" s="22"/>
-      <c r="J62" s="22"/>
-      <c r="K62" s="22"/>
-      <c r="L62" s="22"/>
-      <c r="M62" s="23"/>
+      <c r="I62" s="20"/>
+      <c r="J62" s="20"/>
+      <c r="K62" s="20"/>
+      <c r="L62" s="20"/>
+      <c r="M62" s="21"/>
     </row>
     <row r="63" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="I63" s="22"/>
-      <c r="J63" s="22"/>
-      <c r="K63" s="22"/>
-      <c r="L63" s="22"/>
-      <c r="M63" s="23"/>
+      <c r="I63" s="20"/>
+      <c r="J63" s="20"/>
+      <c r="K63" s="20"/>
+      <c r="L63" s="20"/>
+      <c r="M63" s="21"/>
     </row>
     <row r="64" spans="9:13" x14ac:dyDescent="0.25">
-      <c r="L64" s="22" t="str" cm="1">
+      <c r="L64" s="20" t="str" cm="1">
         <f t="array" ref="L64">IF($G64="","",
   _xlfn.LET(
     _xlpm.topic,$G64,
@@ -3632,7 +3663,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M64" s="23" t="str" cm="1">
+      <c r="M64" s="21" t="str" cm="1">
         <f t="array" ref="M64">IF($G64="","",
   _xlfn.LET(
     _xlpm.topic,$G64,
@@ -3652,7 +3683,7 @@
       </c>
     </row>
     <row r="65" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L65" s="22" t="str" cm="1">
+      <c r="L65" s="20" t="str" cm="1">
         <f t="array" ref="L65">IF($G65="","",
   _xlfn.LET(
     _xlpm.topic,$G65,
@@ -3670,7 +3701,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M65" s="23" t="str" cm="1">
+      <c r="M65" s="21" t="str" cm="1">
         <f t="array" ref="M65">IF($G65="","",
   _xlfn.LET(
     _xlpm.topic,$G65,
@@ -3690,7 +3721,7 @@
       </c>
     </row>
     <row r="66" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L66" s="22" t="str" cm="1">
+      <c r="L66" s="20" t="str" cm="1">
         <f t="array" ref="L66">IF($G66="","",
   _xlfn.LET(
     _xlpm.topic,$G66,
@@ -3708,7 +3739,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M66" s="23" t="str" cm="1">
+      <c r="M66" s="21" t="str" cm="1">
         <f t="array" ref="M66">IF($G66="","",
   _xlfn.LET(
     _xlpm.topic,$G66,
@@ -3728,7 +3759,7 @@
       </c>
     </row>
     <row r="67" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L67" s="22" t="str" cm="1">
+      <c r="L67" s="20" t="str" cm="1">
         <f t="array" ref="L67">IF($G67="","",
   _xlfn.LET(
     _xlpm.topic,$G67,
@@ -3746,7 +3777,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M67" s="23" t="str" cm="1">
+      <c r="M67" s="21" t="str" cm="1">
         <f t="array" ref="M67">IF($G67="","",
   _xlfn.LET(
     _xlpm.topic,$G67,
@@ -3766,7 +3797,7 @@
       </c>
     </row>
     <row r="68" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L68" s="22" t="str" cm="1">
+      <c r="L68" s="20" t="str" cm="1">
         <f t="array" ref="L68">IF($G68="","",
   _xlfn.LET(
     _xlpm.topic,$G68,
@@ -3784,7 +3815,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M68" s="23" t="str" cm="1">
+      <c r="M68" s="21" t="str" cm="1">
         <f t="array" ref="M68">IF($G68="","",
   _xlfn.LET(
     _xlpm.topic,$G68,
@@ -3804,7 +3835,7 @@
       </c>
     </row>
     <row r="69" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L69" s="22" t="str" cm="1">
+      <c r="L69" s="20" t="str" cm="1">
         <f t="array" ref="L69">IF($G69="","",
   _xlfn.LET(
     _xlpm.topic,$G69,
@@ -3822,7 +3853,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M69" s="23" t="str" cm="1">
+      <c r="M69" s="21" t="str" cm="1">
         <f t="array" ref="M69">IF($G69="","",
   _xlfn.LET(
     _xlpm.topic,$G69,
@@ -3842,7 +3873,7 @@
       </c>
     </row>
     <row r="70" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L70" s="22" t="str" cm="1">
+      <c r="L70" s="20" t="str" cm="1">
         <f t="array" ref="L70">IF($G70="","",
   _xlfn.LET(
     _xlpm.topic,$G70,
@@ -3860,7 +3891,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M70" s="23" t="str" cm="1">
+      <c r="M70" s="21" t="str" cm="1">
         <f t="array" ref="M70">IF($G70="","",
   _xlfn.LET(
     _xlpm.topic,$G70,
@@ -3880,7 +3911,7 @@
       </c>
     </row>
     <row r="71" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L71" s="22" t="str" cm="1">
+      <c r="L71" s="20" t="str" cm="1">
         <f t="array" ref="L71">IF($G71="","",
   _xlfn.LET(
     _xlpm.topic,$G71,
@@ -3898,7 +3929,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M71" s="23" t="str" cm="1">
+      <c r="M71" s="21" t="str" cm="1">
         <f t="array" ref="M71">IF($G71="","",
   _xlfn.LET(
     _xlpm.topic,$G71,
@@ -3918,7 +3949,7 @@
       </c>
     </row>
     <row r="72" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L72" s="22" t="str" cm="1">
+      <c r="L72" s="20" t="str" cm="1">
         <f t="array" ref="L72">IF($G72="","",
   _xlfn.LET(
     _xlpm.topic,$G72,
@@ -3936,7 +3967,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M72" s="23" t="str" cm="1">
+      <c r="M72" s="21" t="str" cm="1">
         <f t="array" ref="M72">IF($G72="","",
   _xlfn.LET(
     _xlpm.topic,$G72,
@@ -3956,7 +3987,7 @@
       </c>
     </row>
     <row r="73" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L73" s="22" t="str" cm="1">
+      <c r="L73" s="20" t="str" cm="1">
         <f t="array" ref="L73">IF($G73="","",
   _xlfn.LET(
     _xlpm.topic,$G73,
@@ -3974,7 +4005,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M73" s="23" t="str" cm="1">
+      <c r="M73" s="21" t="str" cm="1">
         <f t="array" ref="M73">IF($G73="","",
   _xlfn.LET(
     _xlpm.topic,$G73,
@@ -3994,7 +4025,7 @@
       </c>
     </row>
     <row r="74" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L74" s="22" t="str" cm="1">
+      <c r="L74" s="20" t="str" cm="1">
         <f t="array" ref="L74">IF($G74="","",
   _xlfn.LET(
     _xlpm.topic,$G74,
@@ -4012,7 +4043,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M74" s="23" t="str" cm="1">
+      <c r="M74" s="21" t="str" cm="1">
         <f t="array" ref="M74">IF($G74="","",
   _xlfn.LET(
     _xlpm.topic,$G74,
@@ -4032,7 +4063,7 @@
       </c>
     </row>
     <row r="75" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L75" s="22" t="str" cm="1">
+      <c r="L75" s="20" t="str" cm="1">
         <f t="array" ref="L75">IF($G75="","",
   _xlfn.LET(
     _xlpm.topic,$G75,
@@ -4050,7 +4081,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M75" s="23" t="str" cm="1">
+      <c r="M75" s="21" t="str" cm="1">
         <f t="array" ref="M75">IF($G75="","",
   _xlfn.LET(
     _xlpm.topic,$G75,
@@ -4070,7 +4101,7 @@
       </c>
     </row>
     <row r="76" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L76" s="22" t="str" cm="1">
+      <c r="L76" s="20" t="str" cm="1">
         <f t="array" ref="L76">IF($G76="","",
   _xlfn.LET(
     _xlpm.topic,$G76,
@@ -4088,7 +4119,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M76" s="23" t="str" cm="1">
+      <c r="M76" s="21" t="str" cm="1">
         <f t="array" ref="M76">IF($G76="","",
   _xlfn.LET(
     _xlpm.topic,$G76,
@@ -4108,7 +4139,7 @@
       </c>
     </row>
     <row r="77" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L77" s="22" t="str" cm="1">
+      <c r="L77" s="20" t="str" cm="1">
         <f t="array" ref="L77">IF($G77="","",
   _xlfn.LET(
     _xlpm.topic,$G77,
@@ -4126,7 +4157,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M77" s="23" t="str" cm="1">
+      <c r="M77" s="21" t="str" cm="1">
         <f t="array" ref="M77">IF($G77="","",
   _xlfn.LET(
     _xlpm.topic,$G77,
@@ -4146,7 +4177,7 @@
       </c>
     </row>
     <row r="78" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L78" s="22" t="str" cm="1">
+      <c r="L78" s="20" t="str" cm="1">
         <f t="array" ref="L78">IF($G78="","",
   _xlfn.LET(
     _xlpm.topic,$G78,
@@ -4164,7 +4195,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M78" s="23" t="str" cm="1">
+      <c r="M78" s="21" t="str" cm="1">
         <f t="array" ref="M78">IF($G78="","",
   _xlfn.LET(
     _xlpm.topic,$G78,
@@ -4184,7 +4215,7 @@
       </c>
     </row>
     <row r="79" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L79" s="22" t="str" cm="1">
+      <c r="L79" s="20" t="str" cm="1">
         <f t="array" ref="L79">IF($G79="","",
   _xlfn.LET(
     _xlpm.topic,$G79,
@@ -4202,7 +4233,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M79" s="23" t="str" cm="1">
+      <c r="M79" s="21" t="str" cm="1">
         <f t="array" ref="M79">IF($G79="","",
   _xlfn.LET(
     _xlpm.topic,$G79,
@@ -4222,7 +4253,7 @@
       </c>
     </row>
     <row r="80" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L80" s="22" t="str" cm="1">
+      <c r="L80" s="20" t="str" cm="1">
         <f t="array" ref="L80">IF($G80="","",
   _xlfn.LET(
     _xlpm.topic,$G80,
@@ -4240,7 +4271,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M80" s="23" t="str" cm="1">
+      <c r="M80" s="21" t="str" cm="1">
         <f t="array" ref="M80">IF($G80="","",
   _xlfn.LET(
     _xlpm.topic,$G80,
@@ -4260,7 +4291,7 @@
       </c>
     </row>
     <row r="81" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L81" s="22" t="str" cm="1">
+      <c r="L81" s="20" t="str" cm="1">
         <f t="array" ref="L81">IF($G81="","",
   _xlfn.LET(
     _xlpm.topic,$G81,
@@ -4278,7 +4309,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M81" s="23" t="str" cm="1">
+      <c r="M81" s="21" t="str" cm="1">
         <f t="array" ref="M81">IF($G81="","",
   _xlfn.LET(
     _xlpm.topic,$G81,
@@ -4298,7 +4329,7 @@
       </c>
     </row>
     <row r="82" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L82" s="22" t="str" cm="1">
+      <c r="L82" s="20" t="str" cm="1">
         <f t="array" ref="L82">IF($G82="","",
   _xlfn.LET(
     _xlpm.topic,$G82,
@@ -4316,7 +4347,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M82" s="23" t="str" cm="1">
+      <c r="M82" s="21" t="str" cm="1">
         <f t="array" ref="M82">IF($G82="","",
   _xlfn.LET(
     _xlpm.topic,$G82,
@@ -4336,7 +4367,7 @@
       </c>
     </row>
     <row r="83" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L83" s="22" t="str" cm="1">
+      <c r="L83" s="20" t="str" cm="1">
         <f t="array" ref="L83">IF($G83="","",
   _xlfn.LET(
     _xlpm.topic,$G83,
@@ -4354,7 +4385,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M83" s="23" t="str" cm="1">
+      <c r="M83" s="21" t="str" cm="1">
         <f t="array" ref="M83">IF($G83="","",
   _xlfn.LET(
     _xlpm.topic,$G83,
@@ -4374,7 +4405,7 @@
       </c>
     </row>
     <row r="84" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L84" s="22" t="str" cm="1">
+      <c r="L84" s="20" t="str" cm="1">
         <f t="array" ref="L84">IF($G84="","",
   _xlfn.LET(
     _xlpm.topic,$G84,
@@ -4392,7 +4423,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M84" s="23" t="str" cm="1">
+      <c r="M84" s="21" t="str" cm="1">
         <f t="array" ref="M84">IF($G84="","",
   _xlfn.LET(
     _xlpm.topic,$G84,
@@ -4412,7 +4443,7 @@
       </c>
     </row>
     <row r="85" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L85" s="22" t="str" cm="1">
+      <c r="L85" s="20" t="str" cm="1">
         <f t="array" ref="L85">IF($G85="","",
   _xlfn.LET(
     _xlpm.topic,$G85,
@@ -4430,7 +4461,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M85" s="23" t="str" cm="1">
+      <c r="M85" s="21" t="str" cm="1">
         <f t="array" ref="M85">IF($G85="","",
   _xlfn.LET(
     _xlpm.topic,$G85,
@@ -4450,7 +4481,7 @@
       </c>
     </row>
     <row r="86" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L86" s="22" t="str" cm="1">
+      <c r="L86" s="20" t="str" cm="1">
         <f t="array" ref="L86">IF($G86="","",
   _xlfn.LET(
     _xlpm.topic,$G86,
@@ -4468,7 +4499,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M86" s="23" t="str" cm="1">
+      <c r="M86" s="21" t="str" cm="1">
         <f t="array" ref="M86">IF($G86="","",
   _xlfn.LET(
     _xlpm.topic,$G86,
@@ -4488,7 +4519,7 @@
       </c>
     </row>
     <row r="87" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L87" s="22" t="str" cm="1">
+      <c r="L87" s="20" t="str" cm="1">
         <f t="array" ref="L87">IF($G87="","",
   _xlfn.LET(
     _xlpm.topic,$G87,
@@ -4506,7 +4537,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M87" s="23" t="str" cm="1">
+      <c r="M87" s="21" t="str" cm="1">
         <f t="array" ref="M87">IF($G87="","",
   _xlfn.LET(
     _xlpm.topic,$G87,
@@ -4526,7 +4557,7 @@
       </c>
     </row>
     <row r="88" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L88" s="22" t="str" cm="1">
+      <c r="L88" s="20" t="str" cm="1">
         <f t="array" ref="L88">IF($G88="","",
   _xlfn.LET(
     _xlpm.topic,$G88,
@@ -4544,7 +4575,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M88" s="23" t="str" cm="1">
+      <c r="M88" s="21" t="str" cm="1">
         <f t="array" ref="M88">IF($G88="","",
   _xlfn.LET(
     _xlpm.topic,$G88,
@@ -4564,7 +4595,7 @@
       </c>
     </row>
     <row r="89" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L89" s="22" t="str" cm="1">
+      <c r="L89" s="20" t="str" cm="1">
         <f t="array" ref="L89">IF($G89="","",
   _xlfn.LET(
     _xlpm.topic,$G89,
@@ -4582,7 +4613,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M89" s="23" t="str" cm="1">
+      <c r="M89" s="21" t="str" cm="1">
         <f t="array" ref="M89">IF($G89="","",
   _xlfn.LET(
     _xlpm.topic,$G89,
@@ -4602,7 +4633,7 @@
       </c>
     </row>
     <row r="90" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L90" s="22" t="str" cm="1">
+      <c r="L90" s="20" t="str" cm="1">
         <f t="array" ref="L90">IF($G90="","",
   _xlfn.LET(
     _xlpm.topic,$G90,
@@ -4620,7 +4651,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M90" s="23" t="str" cm="1">
+      <c r="M90" s="21" t="str" cm="1">
         <f t="array" ref="M90">IF($G90="","",
   _xlfn.LET(
     _xlpm.topic,$G90,
@@ -4640,7 +4671,7 @@
       </c>
     </row>
     <row r="91" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L91" s="22" t="str" cm="1">
+      <c r="L91" s="20" t="str" cm="1">
         <f t="array" ref="L91">IF($G91="","",
   _xlfn.LET(
     _xlpm.topic,$G91,
@@ -4658,7 +4689,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M91" s="23" t="str" cm="1">
+      <c r="M91" s="21" t="str" cm="1">
         <f t="array" ref="M91">IF($G91="","",
   _xlfn.LET(
     _xlpm.topic,$G91,
@@ -4678,7 +4709,7 @@
       </c>
     </row>
     <row r="92" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L92" s="22" t="str" cm="1">
+      <c r="L92" s="20" t="str" cm="1">
         <f t="array" ref="L92">IF($G92="","",
   _xlfn.LET(
     _xlpm.topic,$G92,
@@ -4696,7 +4727,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M92" s="23" t="str" cm="1">
+      <c r="M92" s="21" t="str" cm="1">
         <f t="array" ref="M92">IF($G92="","",
   _xlfn.LET(
     _xlpm.topic,$G92,
@@ -4716,7 +4747,7 @@
       </c>
     </row>
     <row r="93" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L93" s="22" t="str" cm="1">
+      <c r="L93" s="20" t="str" cm="1">
         <f t="array" ref="L93">IF($G93="","",
   _xlfn.LET(
     _xlpm.topic,$G93,
@@ -4734,7 +4765,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M93" s="23" t="str" cm="1">
+      <c r="M93" s="21" t="str" cm="1">
         <f t="array" ref="M93">IF($G93="","",
   _xlfn.LET(
     _xlpm.topic,$G93,
@@ -4754,7 +4785,7 @@
       </c>
     </row>
     <row r="94" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L94" s="22" t="str" cm="1">
+      <c r="L94" s="20" t="str" cm="1">
         <f t="array" ref="L94">IF($G94="","",
   _xlfn.LET(
     _xlpm.topic,$G94,
@@ -4772,7 +4803,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M94" s="23" t="str" cm="1">
+      <c r="M94" s="21" t="str" cm="1">
         <f t="array" ref="M94">IF($G94="","",
   _xlfn.LET(
     _xlpm.topic,$G94,
@@ -4792,7 +4823,7 @@
       </c>
     </row>
     <row r="95" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L95" s="22" t="str" cm="1">
+      <c r="L95" s="20" t="str" cm="1">
         <f t="array" ref="L95">IF($G95="","",
   _xlfn.LET(
     _xlpm.topic,$G95,
@@ -4810,7 +4841,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M95" s="23" t="str" cm="1">
+      <c r="M95" s="21" t="str" cm="1">
         <f t="array" ref="M95">IF($G95="","",
   _xlfn.LET(
     _xlpm.topic,$G95,
@@ -4830,7 +4861,7 @@
       </c>
     </row>
     <row r="96" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L96" s="22" t="str" cm="1">
+      <c r="L96" s="20" t="str" cm="1">
         <f t="array" ref="L96">IF($G96="","",
   _xlfn.LET(
     _xlpm.topic,$G96,
@@ -4848,7 +4879,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M96" s="23" t="str" cm="1">
+      <c r="M96" s="21" t="str" cm="1">
         <f t="array" ref="M96">IF($G96="","",
   _xlfn.LET(
     _xlpm.topic,$G96,
@@ -4868,7 +4899,7 @@
       </c>
     </row>
     <row r="97" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L97" s="22" t="str" cm="1">
+      <c r="L97" s="20" t="str" cm="1">
         <f t="array" ref="L97">IF($G97="","",
   _xlfn.LET(
     _xlpm.topic,$G97,
@@ -4886,7 +4917,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M97" s="23" t="str" cm="1">
+      <c r="M97" s="21" t="str" cm="1">
         <f t="array" ref="M97">IF($G97="","",
   _xlfn.LET(
     _xlpm.topic,$G97,
@@ -4906,7 +4937,7 @@
       </c>
     </row>
     <row r="98" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L98" s="22" t="str" cm="1">
+      <c r="L98" s="20" t="str" cm="1">
         <f t="array" ref="L98">IF($G98="","",
   _xlfn.LET(
     _xlpm.topic,$G98,
@@ -4924,7 +4955,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M98" s="23" t="str" cm="1">
+      <c r="M98" s="21" t="str" cm="1">
         <f t="array" ref="M98">IF($G98="","",
   _xlfn.LET(
     _xlpm.topic,$G98,
@@ -4944,7 +4975,7 @@
       </c>
     </row>
     <row r="99" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L99" s="22" t="str" cm="1">
+      <c r="L99" s="20" t="str" cm="1">
         <f t="array" ref="L99">IF($G99="","",
   _xlfn.LET(
     _xlpm.topic,$G99,
@@ -4962,7 +4993,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M99" s="23" t="str" cm="1">
+      <c r="M99" s="21" t="str" cm="1">
         <f t="array" ref="M99">IF($G99="","",
   _xlfn.LET(
     _xlpm.topic,$G99,
@@ -4982,7 +5013,7 @@
       </c>
     </row>
     <row r="100" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L100" s="22" t="str" cm="1">
+      <c r="L100" s="20" t="str" cm="1">
         <f t="array" ref="L100">IF($G100="","",
   _xlfn.LET(
     _xlpm.topic,$G100,
@@ -5000,7 +5031,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M100" s="23" t="str" cm="1">
+      <c r="M100" s="21" t="str" cm="1">
         <f t="array" ref="M100">IF($G100="","",
   _xlfn.LET(
     _xlpm.topic,$G100,
@@ -5020,7 +5051,7 @@
       </c>
     </row>
     <row r="101" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L101" s="22" t="str" cm="1">
+      <c r="L101" s="20" t="str" cm="1">
         <f t="array" ref="L101">IF($G101="","",
   _xlfn.LET(
     _xlpm.topic,$G101,
@@ -5038,7 +5069,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M101" s="23" t="str" cm="1">
+      <c r="M101" s="21" t="str" cm="1">
         <f t="array" ref="M101">IF($G101="","",
   _xlfn.LET(
     _xlpm.topic,$G101,
@@ -5058,7 +5089,7 @@
       </c>
     </row>
     <row r="102" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L102" s="22" t="str" cm="1">
+      <c r="L102" s="20" t="str" cm="1">
         <f t="array" ref="L102">IF($G102="","",
   _xlfn.LET(
     _xlpm.topic,$G102,
@@ -5076,7 +5107,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M102" s="23" t="str" cm="1">
+      <c r="M102" s="21" t="str" cm="1">
         <f t="array" ref="M102">IF($G102="","",
   _xlfn.LET(
     _xlpm.topic,$G102,
@@ -5096,7 +5127,7 @@
       </c>
     </row>
     <row r="103" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L103" s="22" t="str" cm="1">
+      <c r="L103" s="20" t="str" cm="1">
         <f t="array" ref="L103">IF($G103="","",
   _xlfn.LET(
     _xlpm.topic,$G103,
@@ -5114,7 +5145,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M103" s="23" t="str" cm="1">
+      <c r="M103" s="21" t="str" cm="1">
         <f t="array" ref="M103">IF($G103="","",
   _xlfn.LET(
     _xlpm.topic,$G103,
@@ -5134,7 +5165,7 @@
       </c>
     </row>
     <row r="104" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L104" s="22" t="str" cm="1">
+      <c r="L104" s="20" t="str" cm="1">
         <f t="array" ref="L104">IF($G104="","",
   _xlfn.LET(
     _xlpm.topic,$G104,
@@ -5152,7 +5183,7 @@
 )</f>
         <v/>
       </c>
-      <c r="M104" s="23" t="str" cm="1">
+      <c r="M104" s="21" t="str" cm="1">
         <f t="array" ref="M104">IF($G104="","",
   _xlfn.LET(
     _xlpm.topic,$G104,

</xml_diff>